<commit_message>
Add guest reporting feature and update report files
</commit_message>
<xml_diff>
--- a/outputs/final-report/HMMS_FULL_TEST_CASES.xlsx
+++ b/outputs/final-report/HMMS_FULL_TEST_CASES.xlsx
@@ -2,25 +2,28 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEST SUMMARY" sheetId="1" r:id="Rd0df8aae689e4249"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-001" sheetId="2" r:id="Rb3765462a2dd4f59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-002" sheetId="3" r:id="Rea684a20695a40ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-003" sheetId="4" r:id="R11ca3e8251b14d51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-004" sheetId="5" r:id="R38e0c234ab18413b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-005" sheetId="6" r:id="R6aa7e95e09084fc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-006" sheetId="7" r:id="Rddb21c434e7b4532"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-007" sheetId="8" r:id="Rf7b7f5107f8b4558"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-008" sheetId="9" r:id="R2e4ac9165c0f413a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-009" sheetId="10" r:id="Red10e98b21ee4bc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-010" sheetId="11" r:id="R07c612290742488c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-011" sheetId="12" r:id="R5e11953eb83047a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-012" sheetId="13" r:id="Ra5e3cde8b33e4e86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-013" sheetId="14" r:id="R8529e96f04bc4287"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-014" sheetId="15" r:id="Rc172e16f7c614f89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-015" sheetId="16" r:id="R0e032c7a377f4d58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-016" sheetId="17" r:id="R8e455d1068934bd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-017" sheetId="18" r:id="R96f485475f754be5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-018" sheetId="19" r:id="R614fcda0b7b54522"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEST SUMMARY" sheetId="1" r:id="R38ea3c5266bc465a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-001" sheetId="2" r:id="R5d96b926092b4ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-002" sheetId="3" r:id="R04ce38be31004e3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-003" sheetId="4" r:id="R5a401b0f35bd4b56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-004" sheetId="5" r:id="Rb1b47d9c35ca4ca3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-005" sheetId="6" r:id="Rea4100992cd24e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-006" sheetId="7" r:id="Red1e150b748f49b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-007" sheetId="8" r:id="Rb2e5482a1123400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-008" sheetId="9" r:id="Rc747a17ae99a4620"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-009" sheetId="10" r:id="Rf185db9ec6e1496b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-010" sheetId="11" r:id="Rfcd5e24bc9354062"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-011" sheetId="12" r:id="Raedffbb03cbe41dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-012" sheetId="13" r:id="Ra82f6189558145c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-013" sheetId="14" r:id="Rcacd9cfa61044e47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-014" sheetId="15" r:id="Rb223ff893b7b4c19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-015" sheetId="16" r:id="R70243905a7c44313"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-016" sheetId="17" r:id="Rcdaf47c6cc504a92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-017" sheetId="18" r:id="R467d3770706742a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-018" sheetId="19" r:id="R0b5d6e16152c4677"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-019" sheetId="20" r:id="R37e476fe827a4a4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-020" sheetId="21" r:id="Rbec0cf09fe1c4c57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC-021" sheetId="22" r:id="R702b4fcd0be84fc4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -488,7 +491,7 @@
         <x:v>Total Test Cases</x:v>
       </x:c>
       <x:c r="B4" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D4" s="17" t="str">
         <x:v>TC-001</x:v>
@@ -511,7 +514,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="B5" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D5" s="17" t="str">
         <x:v>TC-002</x:v>
@@ -801,15 +804,66 @@
         <x:v>TC-018</x:v>
       </x:c>
       <x:c r="E21" s="17" t="str">
+        <x:v>Guest Access</x:v>
+      </x:c>
+      <x:c r="F21" s="17" t="str">
+        <x:v>Continue as Guest from login page</x:v>
+      </x:c>
+      <x:c r="G21" s="18" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H21" s="17" t="str">
+        <x:v>Execution record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="D22" s="17" t="str">
+        <x:v>TC-019</x:v>
+      </x:c>
+      <x:c r="E22" s="17" t="str">
+        <x:v>Guest Report</x:v>
+      </x:c>
+      <x:c r="F22" s="17" t="str">
+        <x:v>Submit guest maintenance report with image</x:v>
+      </x:c>
+      <x:c r="G22" s="18" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H22" s="17" t="str">
+        <x:v>Execution record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="D23" s="17" t="str">
+        <x:v>TC-020</x:v>
+      </x:c>
+      <x:c r="E23" s="17" t="str">
+        <x:v>Guest Security</x:v>
+      </x:c>
+      <x:c r="F23" s="17" t="str">
+        <x:v>Guest cannot view protected maintenance pages</x:v>
+      </x:c>
+      <x:c r="G23" s="18" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H23" s="17" t="str">
+        <x:v>Execution record</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="D24" s="17" t="str">
+        <x:v>TC-021</x:v>
+      </x:c>
+      <x:c r="E24" s="17" t="str">
         <x:v>Technical Validation</x:v>
       </x:c>
-      <x:c r="F21" s="17" t="str">
+      <x:c r="F24" s="17" t="str">
         <x:v>Automated regression suite</x:v>
       </x:c>
-      <x:c r="G21" s="18" t="str">
-        <x:v>Pass</x:v>
-      </x:c>
-      <x:c r="H21" s="17" t="str">
+      <x:c r="G24" s="18" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H24" s="17" t="str">
         <x:v>Execution record</x:v>
       </x:c>
     </x:row>
@@ -3243,7 +3297,7 @@
       </x:c>
       <x:c r="E1" s="25"/>
       <x:c r="F1" s="22" t="str">
-        <x:v>Automated regression suite</x:v>
+        <x:v>Continue as Guest from login page</x:v>
       </x:c>
       <x:c r="G1" s="22"/>
       <x:c r="H1" s="22"/>
@@ -3314,7 +3368,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="22" t="str">
-        <x:v>PHPUnit feature and unit tests</x:v>
+        <x:v>Unauthenticated browser session</x:v>
       </x:c>
       <x:c r="H5" s="22"/>
       <x:c r="I5" s="22"/>
@@ -3343,7 +3397,7 @@
         <x:v>Test Scenario</x:v>
       </x:c>
       <x:c r="B7" s="27" t="str">
-        <x:v>Automated regression suite</x:v>
+        <x:v>Continue as Guest from login page</x:v>
       </x:c>
       <x:c r="C7" s="27"/>
       <x:c r="D7" s="27"/>
@@ -3390,12 +3444,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B10" s="22" t="str">
-        <x:v>Run the project test suite</x:v>
+        <x:v>Open the login page</x:v>
       </x:c>
       <x:c r="C10" s="22"/>
       <x:c r="D10" s="22"/>
       <x:c r="E10" s="22" t="str">
-        <x:v>Test runner starts without configuration error</x:v>
+        <x:v>Login page is displayed</x:v>
       </x:c>
       <x:c r="F10" s="22"/>
       <x:c r="G10" s="22" t="str">
@@ -3411,12 +3465,12 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
-        <x:v>Review all test groups</x:v>
+        <x:v>Select Continue as Guest</x:v>
       </x:c>
       <x:c r="C11" s="22"/>
       <x:c r="D11" s="22"/>
       <x:c r="E11" s="22" t="str">
-        <x:v>Authentication, profile and application tests complete</x:v>
+        <x:v>Guest option is visible and clickable</x:v>
       </x:c>
       <x:c r="F11" s="22"/>
       <x:c r="G11" s="22" t="str">
@@ -3432,12 +3486,12 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B12" s="22" t="str">
-        <x:v>Confirm assertion summary</x:v>
+        <x:v>Observe the guest report page</x:v>
       </x:c>
       <x:c r="C12" s="22"/>
       <x:c r="D12" s="22"/>
       <x:c r="E12" s="22" t="str">
-        <x:v>25 tests and 62 assertions pass with zero failures</x:v>
+        <x:v>Guest Maintenance Report page opens without authentication</x:v>
       </x:c>
       <x:c r="F12" s="22"/>
       <x:c r="G12" s="22" t="str">
@@ -3747,6 +3801,804 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="25" t="str">
+        <x:v>Test Case ID</x:v>
+      </x:c>
+      <x:c r="B1" s="25"/>
+      <x:c r="C1" s="22" t="str">
+        <x:v>TC-019</x:v>
+      </x:c>
+      <x:c r="D1" s="25" t="str">
+        <x:v>Test Case Description</x:v>
+      </x:c>
+      <x:c r="E1" s="25"/>
+      <x:c r="F1" s="22" t="str">
+        <x:v>Submit guest maintenance report with image</x:v>
+      </x:c>
+      <x:c r="G1" s="22"/>
+      <x:c r="H1" s="22"/>
+      <x:c r="I1" s="22"/>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="25" t="str">
+        <x:v>Version</x:v>
+      </x:c>
+      <x:c r="B2" s="25"/>
+      <x:c r="C2" s="22" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="D2" s="25" t="str">
+        <x:v>Date Tested</x:v>
+      </x:c>
+      <x:c r="E2" s="25"/>
+      <x:c r="F2" s="31" t="n">
+        <x:v>46204</x:v>
+      </x:c>
+      <x:c r="G2" s="31"/>
+      <x:c r="H2" s="25" t="str">
+        <x:v>Status: Pass</x:v>
+      </x:c>
+      <x:c r="I2" s="25"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="21"/>
+      <x:c r="B3" s="21"/>
+      <x:c r="C3" s="21"/>
+      <x:c r="D3" s="21"/>
+      <x:c r="E3" s="21"/>
+      <x:c r="F3" s="21"/>
+      <x:c r="G3" s="21"/>
+      <x:c r="H3" s="21"/>
+      <x:c r="I3" s="21"/>
+    </x:row>
+    <x:row r="4" ht="27" customHeight="1">
+      <x:c r="A4" s="25" t="str">
+        <x:v>S #</x:v>
+      </x:c>
+      <x:c r="B4" s="25" t="str">
+        <x:v>Prerequisites</x:v>
+      </x:c>
+      <x:c r="C4" s="25"/>
+      <x:c r="D4" s="25"/>
+      <x:c r="E4" s="25"/>
+      <x:c r="F4" s="25" t="str">
+        <x:v>S #</x:v>
+      </x:c>
+      <x:c r="G4" s="25" t="str">
+        <x:v>Test Data</x:v>
+      </x:c>
+      <x:c r="H4" s="25"/>
+      <x:c r="I4" s="25"/>
+    </x:row>
+    <x:row r="5" ht="27" customHeight="1">
+      <x:c r="A5" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>Application running at http://127.0.0.1:8000</x:v>
+      </x:c>
+      <x:c r="C5" s="22"/>
+      <x:c r="D5" s="22"/>
+      <x:c r="E5" s="22"/>
+      <x:c r="F5" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G5" s="22" t="str">
+        <x:v>Problem title, location, urgency, description and optional image</x:v>
+      </x:c>
+      <x:c r="H5" s="22"/>
+      <x:c r="I5" s="22"/>
+    </x:row>
+    <x:row r="6" ht="27" customHeight="1">
+      <x:c r="A6" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>Supported browser and appropriate test account</x:v>
+      </x:c>
+      <x:c r="C6" s="22"/>
+      <x:c r="D6" s="22"/>
+      <x:c r="E6" s="22"/>
+      <x:c r="F6" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G6" s="22" t="str">
+        <x:v>Seeded local test database</x:v>
+      </x:c>
+      <x:c r="H6" s="22"/>
+      <x:c r="I6" s="22"/>
+    </x:row>
+    <x:row r="7" ht="27" customHeight="1">
+      <x:c r="A7" s="25" t="str">
+        <x:v>Test Scenario</x:v>
+      </x:c>
+      <x:c r="B7" s="27" t="str">
+        <x:v>Submit guest maintenance report with image</x:v>
+      </x:c>
+      <x:c r="C7" s="27"/>
+      <x:c r="D7" s="27"/>
+      <x:c r="E7" s="27"/>
+      <x:c r="F7" s="27"/>
+      <x:c r="G7" s="27"/>
+      <x:c r="H7" s="27"/>
+      <x:c r="I7" s="27"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="21"/>
+      <x:c r="B8" s="21"/>
+      <x:c r="C8" s="21"/>
+      <x:c r="D8" s="21"/>
+      <x:c r="E8" s="21"/>
+      <x:c r="F8" s="21"/>
+      <x:c r="G8" s="21"/>
+      <x:c r="H8" s="21"/>
+      <x:c r="I8" s="21"/>
+    </x:row>
+    <x:row r="9" ht="40" customHeight="1">
+      <x:c r="A9" s="25" t="str">
+        <x:v>Step #</x:v>
+      </x:c>
+      <x:c r="B9" s="25" t="str">
+        <x:v>Step Details</x:v>
+      </x:c>
+      <x:c r="C9" s="25"/>
+      <x:c r="D9" s="25"/>
+      <x:c r="E9" s="25" t="str">
+        <x:v>Expected Results</x:v>
+      </x:c>
+      <x:c r="F9" s="25"/>
+      <x:c r="G9" s="25" t="str">
+        <x:v>Actual Results</x:v>
+      </x:c>
+      <x:c r="H9" s="25"/>
+      <x:c r="I9" s="25" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="40" customHeight="1">
+      <x:c r="A10" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>Open the guest report page</x:v>
+      </x:c>
+      <x:c r="C10" s="22"/>
+      <x:c r="D10" s="22"/>
+      <x:c r="E10" s="22" t="str">
+        <x:v>Guest form is displayed</x:v>
+      </x:c>
+      <x:c r="F10" s="22"/>
+      <x:c r="G10" s="22" t="str">
+        <x:v>As expected</x:v>
+      </x:c>
+      <x:c r="H10" s="22"/>
+      <x:c r="I10" s="30" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="40" customHeight="1">
+      <x:c r="A11" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>Enter issue details and attach a valid image</x:v>
+      </x:c>
+      <x:c r="C11" s="22"/>
+      <x:c r="D11" s="22"/>
+      <x:c r="E11" s="22" t="str">
+        <x:v>Valid guest data and image are accepted</x:v>
+      </x:c>
+      <x:c r="F11" s="22"/>
+      <x:c r="G11" s="22" t="str">
+        <x:v>As expected</x:v>
+      </x:c>
+      <x:c r="H11" s="22"/>
+      <x:c r="I11" s="30" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="40" customHeight="1">
+      <x:c r="A12" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>Submit the guest report</x:v>
+      </x:c>
+      <x:c r="C12" s="22"/>
+      <x:c r="D12" s="22"/>
+      <x:c r="E12" s="22" t="str">
+        <x:v>Report is saved as Pending and success feedback appears</x:v>
+      </x:c>
+      <x:c r="F12" s="22"/>
+      <x:c r="G12" s="22" t="str">
+        <x:v>As expected</x:v>
+      </x:c>
+      <x:c r="H12" s="22"/>
+      <x:c r="I12" s="30" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:B1"/>
+    <x:mergeCell ref="D1:E1"/>
+    <x:mergeCell ref="F1:I1"/>
+    <x:mergeCell ref="A2:B2"/>
+    <x:mergeCell ref="D2:E2"/>
+    <x:mergeCell ref="F2:G2"/>
+    <x:mergeCell ref="H2:I2"/>
+    <x:mergeCell ref="B4:E4"/>
+    <x:mergeCell ref="G4:I4"/>
+    <x:mergeCell ref="B5:E5"/>
+    <x:mergeCell ref="B6:E6"/>
+    <x:mergeCell ref="G5:I5"/>
+    <x:mergeCell ref="G6:I6"/>
+    <x:mergeCell ref="B7:I7"/>
+    <x:mergeCell ref="B9:D9"/>
+    <x:mergeCell ref="E9:F9"/>
+    <x:mergeCell ref="G9:H9"/>
+    <x:mergeCell ref="B10:D10"/>
+    <x:mergeCell ref="E10:F10"/>
+    <x:mergeCell ref="G10:H10"/>
+    <x:mergeCell ref="B11:D11"/>
+    <x:mergeCell ref="E11:F11"/>
+    <x:mergeCell ref="G11:H11"/>
+    <x:mergeCell ref="B12:D12"/>
+    <x:mergeCell ref="E12:F12"/>
+    <x:mergeCell ref="G12:H12"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="25" t="str">
+        <x:v>Test Case ID</x:v>
+      </x:c>
+      <x:c r="B1" s="25"/>
+      <x:c r="C1" s="22" t="str">
+        <x:v>TC-020</x:v>
+      </x:c>
+      <x:c r="D1" s="25" t="str">
+        <x:v>Test Case Description</x:v>
+      </x:c>
+      <x:c r="E1" s="25"/>
+      <x:c r="F1" s="22" t="str">
+        <x:v>Guest cannot view protected maintenance pages</x:v>
+      </x:c>
+      <x:c r="G1" s="22"/>
+      <x:c r="H1" s="22"/>
+      <x:c r="I1" s="22"/>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="25" t="str">
+        <x:v>Version</x:v>
+      </x:c>
+      <x:c r="B2" s="25"/>
+      <x:c r="C2" s="22" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="D2" s="25" t="str">
+        <x:v>Date Tested</x:v>
+      </x:c>
+      <x:c r="E2" s="25"/>
+      <x:c r="F2" s="31" t="n">
+        <x:v>46204</x:v>
+      </x:c>
+      <x:c r="G2" s="31"/>
+      <x:c r="H2" s="25" t="str">
+        <x:v>Status: Pass</x:v>
+      </x:c>
+      <x:c r="I2" s="25"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="21"/>
+      <x:c r="B3" s="21"/>
+      <x:c r="C3" s="21"/>
+      <x:c r="D3" s="21"/>
+      <x:c r="E3" s="21"/>
+      <x:c r="F3" s="21"/>
+      <x:c r="G3" s="21"/>
+      <x:c r="H3" s="21"/>
+      <x:c r="I3" s="21"/>
+    </x:row>
+    <x:row r="4" ht="27" customHeight="1">
+      <x:c r="A4" s="25" t="str">
+        <x:v>S #</x:v>
+      </x:c>
+      <x:c r="B4" s="25" t="str">
+        <x:v>Prerequisites</x:v>
+      </x:c>
+      <x:c r="C4" s="25"/>
+      <x:c r="D4" s="25"/>
+      <x:c r="E4" s="25"/>
+      <x:c r="F4" s="25" t="str">
+        <x:v>S #</x:v>
+      </x:c>
+      <x:c r="G4" s="25" t="str">
+        <x:v>Test Data</x:v>
+      </x:c>
+      <x:c r="H4" s="25"/>
+      <x:c r="I4" s="25"/>
+    </x:row>
+    <x:row r="5" ht="27" customHeight="1">
+      <x:c r="A5" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>Application running at http://127.0.0.1:8000</x:v>
+      </x:c>
+      <x:c r="C5" s="22"/>
+      <x:c r="D5" s="22"/>
+      <x:c r="E5" s="22"/>
+      <x:c r="F5" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G5" s="22" t="str">
+        <x:v>Unauthenticated guest session</x:v>
+      </x:c>
+      <x:c r="H5" s="22"/>
+      <x:c r="I5" s="22"/>
+    </x:row>
+    <x:row r="6" ht="27" customHeight="1">
+      <x:c r="A6" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>Supported browser and appropriate test account</x:v>
+      </x:c>
+      <x:c r="C6" s="22"/>
+      <x:c r="D6" s="22"/>
+      <x:c r="E6" s="22"/>
+      <x:c r="F6" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G6" s="22" t="str">
+        <x:v>Seeded local test database</x:v>
+      </x:c>
+      <x:c r="H6" s="22"/>
+      <x:c r="I6" s="22"/>
+    </x:row>
+    <x:row r="7" ht="27" customHeight="1">
+      <x:c r="A7" s="25" t="str">
+        <x:v>Test Scenario</x:v>
+      </x:c>
+      <x:c r="B7" s="27" t="str">
+        <x:v>Guest cannot view protected maintenance pages</x:v>
+      </x:c>
+      <x:c r="C7" s="27"/>
+      <x:c r="D7" s="27"/>
+      <x:c r="E7" s="27"/>
+      <x:c r="F7" s="27"/>
+      <x:c r="G7" s="27"/>
+      <x:c r="H7" s="27"/>
+      <x:c r="I7" s="27"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="21"/>
+      <x:c r="B8" s="21"/>
+      <x:c r="C8" s="21"/>
+      <x:c r="D8" s="21"/>
+      <x:c r="E8" s="21"/>
+      <x:c r="F8" s="21"/>
+      <x:c r="G8" s="21"/>
+      <x:c r="H8" s="21"/>
+      <x:c r="I8" s="21"/>
+    </x:row>
+    <x:row r="9" ht="40" customHeight="1">
+      <x:c r="A9" s="25" t="str">
+        <x:v>Step #</x:v>
+      </x:c>
+      <x:c r="B9" s="25" t="str">
+        <x:v>Step Details</x:v>
+      </x:c>
+      <x:c r="C9" s="25"/>
+      <x:c r="D9" s="25"/>
+      <x:c r="E9" s="25" t="str">
+        <x:v>Expected Results</x:v>
+      </x:c>
+      <x:c r="F9" s="25"/>
+      <x:c r="G9" s="25" t="str">
+        <x:v>Actual Results</x:v>
+      </x:c>
+      <x:c r="H9" s="25"/>
+      <x:c r="I9" s="25" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="40" customHeight="1">
+      <x:c r="A10" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>Submit or open guest report page</x:v>
+      </x:c>
+      <x:c r="C10" s="22"/>
+      <x:c r="D10" s="22"/>
+      <x:c r="E10" s="22" t="str">
+        <x:v>Guest report page remains public</x:v>
+      </x:c>
+      <x:c r="F10" s="22"/>
+      <x:c r="G10" s="22" t="str">
+        <x:v>As expected</x:v>
+      </x:c>
+      <x:c r="H10" s="22"/>
+      <x:c r="I10" s="30" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="40" customHeight="1">
+      <x:c r="A11" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>Navigate directly to /dashboard</x:v>
+      </x:c>
+      <x:c r="C11" s="22"/>
+      <x:c r="D11" s="22"/>
+      <x:c r="E11" s="22" t="str">
+        <x:v>Dashboard redirects to Login</x:v>
+      </x:c>
+      <x:c r="F11" s="22"/>
+      <x:c r="G11" s="22" t="str">
+        <x:v>As expected</x:v>
+      </x:c>
+      <x:c r="H11" s="22"/>
+      <x:c r="I11" s="30" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="40" customHeight="1">
+      <x:c r="A12" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>Navigate directly to /maintenance</x:v>
+      </x:c>
+      <x:c r="C12" s="22"/>
+      <x:c r="D12" s="22"/>
+      <x:c r="E12" s="22" t="str">
+        <x:v>Maintenance list redirects to Login</x:v>
+      </x:c>
+      <x:c r="F12" s="22"/>
+      <x:c r="G12" s="22" t="str">
+        <x:v>As expected</x:v>
+      </x:c>
+      <x:c r="H12" s="22"/>
+      <x:c r="I12" s="30" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:B1"/>
+    <x:mergeCell ref="D1:E1"/>
+    <x:mergeCell ref="F1:I1"/>
+    <x:mergeCell ref="A2:B2"/>
+    <x:mergeCell ref="D2:E2"/>
+    <x:mergeCell ref="F2:G2"/>
+    <x:mergeCell ref="H2:I2"/>
+    <x:mergeCell ref="B4:E4"/>
+    <x:mergeCell ref="G4:I4"/>
+    <x:mergeCell ref="B5:E5"/>
+    <x:mergeCell ref="B6:E6"/>
+    <x:mergeCell ref="G5:I5"/>
+    <x:mergeCell ref="G6:I6"/>
+    <x:mergeCell ref="B7:I7"/>
+    <x:mergeCell ref="B9:D9"/>
+    <x:mergeCell ref="E9:F9"/>
+    <x:mergeCell ref="G9:H9"/>
+    <x:mergeCell ref="B10:D10"/>
+    <x:mergeCell ref="E10:F10"/>
+    <x:mergeCell ref="G10:H10"/>
+    <x:mergeCell ref="B11:D11"/>
+    <x:mergeCell ref="E11:F11"/>
+    <x:mergeCell ref="G11:H11"/>
+    <x:mergeCell ref="B12:D12"/>
+    <x:mergeCell ref="E12:F12"/>
+    <x:mergeCell ref="G12:H12"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="25" t="str">
+        <x:v>Test Case ID</x:v>
+      </x:c>
+      <x:c r="B1" s="25"/>
+      <x:c r="C1" s="22" t="str">
+        <x:v>TC-021</x:v>
+      </x:c>
+      <x:c r="D1" s="25" t="str">
+        <x:v>Test Case Description</x:v>
+      </x:c>
+      <x:c r="E1" s="25"/>
+      <x:c r="F1" s="22" t="str">
+        <x:v>Automated regression suite</x:v>
+      </x:c>
+      <x:c r="G1" s="22"/>
+      <x:c r="H1" s="22"/>
+      <x:c r="I1" s="22"/>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="25" t="str">
+        <x:v>Version</x:v>
+      </x:c>
+      <x:c r="B2" s="25"/>
+      <x:c r="C2" s="22" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="D2" s="25" t="str">
+        <x:v>Date Tested</x:v>
+      </x:c>
+      <x:c r="E2" s="25"/>
+      <x:c r="F2" s="31" t="n">
+        <x:v>46204</x:v>
+      </x:c>
+      <x:c r="G2" s="31"/>
+      <x:c r="H2" s="25" t="str">
+        <x:v>Status: Pass</x:v>
+      </x:c>
+      <x:c r="I2" s="25"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="21"/>
+      <x:c r="B3" s="21"/>
+      <x:c r="C3" s="21"/>
+      <x:c r="D3" s="21"/>
+      <x:c r="E3" s="21"/>
+      <x:c r="F3" s="21"/>
+      <x:c r="G3" s="21"/>
+      <x:c r="H3" s="21"/>
+      <x:c r="I3" s="21"/>
+    </x:row>
+    <x:row r="4" ht="27" customHeight="1">
+      <x:c r="A4" s="25" t="str">
+        <x:v>S #</x:v>
+      </x:c>
+      <x:c r="B4" s="25" t="str">
+        <x:v>Prerequisites</x:v>
+      </x:c>
+      <x:c r="C4" s="25"/>
+      <x:c r="D4" s="25"/>
+      <x:c r="E4" s="25"/>
+      <x:c r="F4" s="25" t="str">
+        <x:v>S #</x:v>
+      </x:c>
+      <x:c r="G4" s="25" t="str">
+        <x:v>Test Data</x:v>
+      </x:c>
+      <x:c r="H4" s="25"/>
+      <x:c r="I4" s="25"/>
+    </x:row>
+    <x:row r="5" ht="27" customHeight="1">
+      <x:c r="A5" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>Application running at http://127.0.0.1:8000</x:v>
+      </x:c>
+      <x:c r="C5" s="22"/>
+      <x:c r="D5" s="22"/>
+      <x:c r="E5" s="22"/>
+      <x:c r="F5" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G5" s="22" t="str">
+        <x:v>PHPUnit feature and unit tests</x:v>
+      </x:c>
+      <x:c r="H5" s="22"/>
+      <x:c r="I5" s="22"/>
+    </x:row>
+    <x:row r="6" ht="27" customHeight="1">
+      <x:c r="A6" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>Supported browser and appropriate test account</x:v>
+      </x:c>
+      <x:c r="C6" s="22"/>
+      <x:c r="D6" s="22"/>
+      <x:c r="E6" s="22"/>
+      <x:c r="F6" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G6" s="22" t="str">
+        <x:v>Seeded local test database</x:v>
+      </x:c>
+      <x:c r="H6" s="22"/>
+      <x:c r="I6" s="22"/>
+    </x:row>
+    <x:row r="7" ht="27" customHeight="1">
+      <x:c r="A7" s="25" t="str">
+        <x:v>Test Scenario</x:v>
+      </x:c>
+      <x:c r="B7" s="27" t="str">
+        <x:v>Automated regression suite</x:v>
+      </x:c>
+      <x:c r="C7" s="27"/>
+      <x:c r="D7" s="27"/>
+      <x:c r="E7" s="27"/>
+      <x:c r="F7" s="27"/>
+      <x:c r="G7" s="27"/>
+      <x:c r="H7" s="27"/>
+      <x:c r="I7" s="27"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="21"/>
+      <x:c r="B8" s="21"/>
+      <x:c r="C8" s="21"/>
+      <x:c r="D8" s="21"/>
+      <x:c r="E8" s="21"/>
+      <x:c r="F8" s="21"/>
+      <x:c r="G8" s="21"/>
+      <x:c r="H8" s="21"/>
+      <x:c r="I8" s="21"/>
+    </x:row>
+    <x:row r="9" ht="40" customHeight="1">
+      <x:c r="A9" s="25" t="str">
+        <x:v>Step #</x:v>
+      </x:c>
+      <x:c r="B9" s="25" t="str">
+        <x:v>Step Details</x:v>
+      </x:c>
+      <x:c r="C9" s="25"/>
+      <x:c r="D9" s="25"/>
+      <x:c r="E9" s="25" t="str">
+        <x:v>Expected Results</x:v>
+      </x:c>
+      <x:c r="F9" s="25"/>
+      <x:c r="G9" s="25" t="str">
+        <x:v>Actual Results</x:v>
+      </x:c>
+      <x:c r="H9" s="25"/>
+      <x:c r="I9" s="25" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="40" customHeight="1">
+      <x:c r="A10" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>Run the project test suite</x:v>
+      </x:c>
+      <x:c r="C10" s="22"/>
+      <x:c r="D10" s="22"/>
+      <x:c r="E10" s="22" t="str">
+        <x:v>Test runner starts without configuration error</x:v>
+      </x:c>
+      <x:c r="F10" s="22"/>
+      <x:c r="G10" s="22" t="str">
+        <x:v>As expected</x:v>
+      </x:c>
+      <x:c r="H10" s="22"/>
+      <x:c r="I10" s="30" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="40" customHeight="1">
+      <x:c r="A11" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>Review all test groups</x:v>
+      </x:c>
+      <x:c r="C11" s="22"/>
+      <x:c r="D11" s="22"/>
+      <x:c r="E11" s="22" t="str">
+        <x:v>Authentication, profile and application tests complete</x:v>
+      </x:c>
+      <x:c r="F11" s="22"/>
+      <x:c r="G11" s="22" t="str">
+        <x:v>As expected</x:v>
+      </x:c>
+      <x:c r="H11" s="22"/>
+      <x:c r="I11" s="30" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="40" customHeight="1">
+      <x:c r="A12" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>Confirm assertion summary</x:v>
+      </x:c>
+      <x:c r="C12" s="22"/>
+      <x:c r="D12" s="22"/>
+      <x:c r="E12" s="22" t="str">
+        <x:v>26 tests and 65 assertions pass with zero failures</x:v>
+      </x:c>
+      <x:c r="F12" s="22"/>
+      <x:c r="G12" s="22" t="str">
+        <x:v>As expected</x:v>
+      </x:c>
+      <x:c r="H12" s="22"/>
+      <x:c r="I12" s="30" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:B1"/>
+    <x:mergeCell ref="D1:E1"/>
+    <x:mergeCell ref="F1:I1"/>
+    <x:mergeCell ref="A2:B2"/>
+    <x:mergeCell ref="D2:E2"/>
+    <x:mergeCell ref="F2:G2"/>
+    <x:mergeCell ref="H2:I2"/>
+    <x:mergeCell ref="B4:E4"/>
+    <x:mergeCell ref="G4:I4"/>
+    <x:mergeCell ref="B5:E5"/>
+    <x:mergeCell ref="B6:E6"/>
+    <x:mergeCell ref="G5:I5"/>
+    <x:mergeCell ref="G6:I6"/>
+    <x:mergeCell ref="B7:I7"/>
+    <x:mergeCell ref="B9:D9"/>
+    <x:mergeCell ref="E9:F9"/>
+    <x:mergeCell ref="G9:H9"/>
+    <x:mergeCell ref="B10:D10"/>
+    <x:mergeCell ref="E10:F10"/>
+    <x:mergeCell ref="G10:H10"/>
+    <x:mergeCell ref="B11:D11"/>
+    <x:mergeCell ref="E11:F11"/>
+    <x:mergeCell ref="G11:H11"/>
+    <x:mergeCell ref="B12:D12"/>
+    <x:mergeCell ref="E12:F12"/>
+    <x:mergeCell ref="G12:H12"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>

</xml_diff>